<commit_message>
feat: beginner sailing course inquiry
</commit_message>
<xml_diff>
--- a/planning.xlsx
+++ b/planning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\3. KhanhHN\workspace\project\cvs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9D9284-E1DC-485B-AA50-6DC958C6A6EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9465BC0-5694-4B74-9D60-167D2D54774F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5415" yWindow="5415" windowWidth="28800" windowHeight="15435" firstSheet="17" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5415" yWindow="5415" windowWidth="28800" windowHeight="15435" firstSheet="14" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.Planning" sheetId="1" r:id="rId1"/>
@@ -35,11 +35,12 @@
     <sheet name="Joining a Beginner Guitar Group" sheetId="29" r:id="rId20"/>
     <sheet name="Sheet1" sheetId="30" r:id="rId21"/>
     <sheet name="Sheet3" sheetId="31" r:id="rId22"/>
-    <sheet name="3.Interview" sheetId="5" r:id="rId23"/>
-    <sheet name="P&amp;C Review 1.0.0" sheetId="6" r:id="rId24"/>
-    <sheet name="P&amp;C Review 1.0.1" sheetId="7" r:id="rId25"/>
-    <sheet name="P&amp;C Review 1.0.2" sheetId="8" r:id="rId26"/>
-    <sheet name="Learning English's Objective" sheetId="13" r:id="rId27"/>
+    <sheet name="Sheet4" sheetId="32" r:id="rId23"/>
+    <sheet name="3.Interview" sheetId="5" r:id="rId24"/>
+    <sheet name="P&amp;C Review 1.0.0" sheetId="6" r:id="rId25"/>
+    <sheet name="P&amp;C Review 1.0.1" sheetId="7" r:id="rId26"/>
+    <sheet name="P&amp;C Review 1.0.2" sheetId="8" r:id="rId27"/>
+    <sheet name="Learning English's Objective" sheetId="13" r:id="rId28"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1708" uniqueCount="1592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1772" uniqueCount="1651">
   <si>
     <t>STT</t>
   </si>
@@ -5099,6 +5100,183 @@
   </si>
   <si>
     <t>Vậy hãy cùng thảo luận…</t>
+  </si>
+  <si>
+    <t>Xin chào, Câu lạc bộ Thuyền buồm Oyster Bay. Tôi có thể giúp gì cho bạn?</t>
+  </si>
+  <si>
+    <t>Ồ chào. Tôi muốn tìm hiểu về các khóa học thuyền buồm cho người mới bắt đầu.</t>
+  </si>
+  <si>
+    <t>Không vấn đề. Khóa học dành cho bạn phải không?</t>
+  </si>
+  <si>
+    <t>Vâng. Tôi đã xem qua trên mạng nhưng tôi không chắc khóa nào là tốt nhất.</t>
+  </si>
+  <si>
+    <t>Được. Có thể bạn sẽ quan tâm đến Ngày Trải Nghiệm của chúng tôi?</t>
+  </si>
+  <si>
+    <t>Có thể.</t>
+  </si>
+  <si>
+    <t>Vâậy những ngày này dành cho những người chưa bao giờ đi thuyền buồm trước đây, về cơ bản là một buổi giới thiệu về thuyền buồm để bạn biết mình có thích nó không và muốn tiếp tục hay không.</t>
+  </si>
+  <si>
+    <t>Và giá của khóa đó là bao nhiêu?</t>
+  </si>
+  <si>
+    <t>Là 120 bảng cho một ngày, những sẽ giảm còn 110 bảng mỗi người nếu có hai người tham gia.</t>
+  </si>
+  <si>
+    <t>Không, chỉ có mình tôi thôi.</t>
+  </si>
+  <si>
+    <t>Ồ, không sao cả.</t>
+  </si>
+  <si>
+    <t>Bạn sẽ học trong một nhóm nhỏ, thường khoảng tám người nhưng không quá mười người và mọi người ở đây đều rất thân thiện.</t>
+  </si>
+  <si>
+    <t>Ừm. Và còn khóa học nào phù hợp khác không?</t>
+  </si>
+  <si>
+    <t>Lựa chọn khác là khóa học Cấp độ 1.</t>
+  </si>
+  <si>
+    <t>Đây là các khóa học kéo dài hai ngày cuối tuần và chúng tôi tổ chức quanh năm.</t>
+  </si>
+  <si>
+    <t>Được. Vậy bạn sẽ học gì trong khóa này?</t>
+  </si>
+  <si>
+    <t>Đây là sự kết hợp giữa lý thuyết và kỹ năng thực hành.</t>
+  </si>
+  <si>
+    <t>Bạn sẽ học về các yếu tố như thời tiết, điều này rõ ràng rất quan trọng và cả thủy triều, cùng các kỹ năng thuyền buồm cơ bản.</t>
+  </si>
+  <si>
+    <t>Bạn sẽ ra cảng trên những thuyền nhỏ huấn luyện đặc biệt dành cho người mới, hai người và một huấn luyện viên trên mỗi chiếc thuyền nhỏ.</t>
+  </si>
+  <si>
+    <t>Huấn luyện viên sẽ đảm bảo bạn hiểu mọi điều cần biết về an toàn.</t>
+  </si>
+  <si>
+    <t>Nghe có vẻ vất vả đấy!</t>
+  </si>
+  <si>
+    <t>Đúng, nhưng bạn cũng sẽ có nhiều niềm vui.</t>
+  </si>
+  <si>
+    <t>Và chi phí của khóa đó là bao nhiêu…?</t>
+  </si>
+  <si>
+    <t>200 bảng.</t>
+  </si>
+  <si>
+    <t>Nhưng sẽ rẻ hơn một chút nếu bạn quyết định tham gia câu lạc bộ.</t>
+  </si>
+  <si>
+    <t>Thành viên sẽ được giảm giá.</t>
+  </si>
+  <si>
+    <t>Tôi vẫn chưa chắc về điều đó.</t>
+  </si>
+  <si>
+    <t>Bạn còn nhiều thời gian để quyết định mà.</t>
+  </si>
+  <si>
+    <t>Và chi phí đó có bao gồm mọi thứ không?</t>
+  </si>
+  <si>
+    <t>Vâng, mọi thứ đều đã bao gồm và bạn cũng sẽ nhận được một cuốn từ điển rất tốt giải thích tất cả các thuật ngữ về chèo thuyền.</t>
+  </si>
+  <si>
+    <t>Rất nhiều người gặp khó khăn với điều này lúc đầu.</t>
+  </si>
+  <si>
+    <t>Trong đó có nhiều hình ảnh, nên tôi chắc chắn bạn sẽ thấy nó rất hữu ích.</t>
+  </si>
+  <si>
+    <t>Và khi hoàn thành khóa học, bạn sẽ nhận được chứng chỉ.</t>
+  </si>
+  <si>
+    <t>Sau đó, bạn sẽ sẵn sàng chuyển sang khóa học Cấp độ 2.</t>
+  </si>
+  <si>
+    <t>Nghe hay đấy.</t>
+  </si>
+  <si>
+    <t>Tôi nghĩ đó là tất cả thông tin bạn cần lúc này.</t>
+  </si>
+  <si>
+    <t>Chỉ còn một vài điều chung chung nữa.</t>
+  </si>
+  <si>
+    <t>Ví dụ, biết bơi là điều thực sự quan trọng.</t>
+  </si>
+  <si>
+    <t>Vâng, tôi khá tự tin khi ở dưới nước.</t>
+  </si>
+  <si>
+    <t>Tuyệt vời.</t>
+  </si>
+  <si>
+    <t>Điều nữa tôi nên nói là chúng tôi cung cấp bộ đồ lặn vào áo phao nhưng bạn cần mang theo quần bơi và một đôi giày thể thao cũ.</t>
+  </si>
+  <si>
+    <t>Còn khăn tắm thì sao?</t>
+  </si>
+  <si>
+    <t>Vâng, chắc chắn rồi.</t>
+  </si>
+  <si>
+    <t>Và bạn cũng có thể muốn mang theo đồ dùng cá nhân, như dầu gội đầu.</t>
+  </si>
+  <si>
+    <t>Còn về đồ ăn thức uống thì sao?</t>
+  </si>
+  <si>
+    <t>Tôi có cần mang theo hay câu lạc bộ có quán cà phê không?</t>
+  </si>
+  <si>
+    <t>Vâng, bạn có thể mua bánh mì sandwich, bánh ngọt và đồ ăn nhẹ ở đó.</t>
+  </si>
+  <si>
+    <t>Đồ ăn ở đó cũng khá hợp lý.</t>
+  </si>
+  <si>
+    <t>Được rồi, tốt quá.</t>
+  </si>
+  <si>
+    <t>Tôi nghĩ mình quan tâm đến khóa học Cấp độ 1.</t>
+  </si>
+  <si>
+    <t>Nhưng tôi hoàn toàn không biết gì về chèo thuyền vậy tôi có thể làm gì để chuẩn bị cho mình một chút không?</t>
+  </si>
+  <si>
+    <t>Tôi khuyên bạn nên xem một số video mà chúng tôi sử dụng cho đào tạo.</t>
+  </si>
+  <si>
+    <t>Chúng có sẵn trên mạng.</t>
+  </si>
+  <si>
+    <t>Tôi có thể gửi cho bạn đường link.</t>
+  </si>
+  <si>
+    <t>Chúng sẽ cho bạn ý tưởng về những gì sẽ diễn ra.</t>
+  </si>
+  <si>
+    <t>Hoàn hảo, cảm ơn. Điều đó sẽ rất hữu ích.</t>
+  </si>
+  <si>
+    <t>Ồ và còn một điều nữa… Tôi sẽ đi xe đạp đến câu lạc bộ và sẽ cần chỗ để cất giữ đồ quý giá.</t>
+  </si>
+  <si>
+    <t>Tôi chỉ muốn hỏi có tủ để đồ cho mọi người không?</t>
+  </si>
+  <si>
+    <t>Vâng, có rất nhiều ở phòng thay đồ.</t>
   </si>
 </sst>
 </file>
@@ -5371,7 +5549,98 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="94">
+  <dxfs count="107">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -8033,7 +8302,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="88" priority="1">
+    <cfRule type="expression" dxfId="101" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8851,7 +9120,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="87" priority="1">
+    <cfRule type="expression" dxfId="100" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9739,7 +10008,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="86" priority="1">
+    <cfRule type="expression" dxfId="99" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10539,7 +10808,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="85" priority="1">
+    <cfRule type="expression" dxfId="98" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11383,7 +11652,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="84" priority="1">
+    <cfRule type="expression" dxfId="97" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12209,7 +12478,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="83" priority="1">
+    <cfRule type="expression" dxfId="96" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12349,7 +12618,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C11">
-    <cfRule type="expression" dxfId="82" priority="1">
+    <cfRule type="expression" dxfId="95" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12623,22 +12892,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C6">
-    <cfRule type="expression" dxfId="81" priority="4">
+    <cfRule type="expression" dxfId="94" priority="4">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A12:C26">
-    <cfRule type="expression" dxfId="80" priority="3">
+    <cfRule type="expression" dxfId="93" priority="3">
       <formula>MOD($A12,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D6">
-    <cfRule type="expression" dxfId="79" priority="2">
+    <cfRule type="expression" dxfId="92" priority="2">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D12:D26">
-    <cfRule type="expression" dxfId="78" priority="1">
+    <cfRule type="expression" dxfId="91" priority="1">
       <formula>MOD($A12,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12888,122 +13157,122 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C8">
-    <cfRule type="expression" dxfId="77" priority="25">
+    <cfRule type="expression" dxfId="90" priority="25">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D8">
-    <cfRule type="expression" dxfId="76" priority="24">
+    <cfRule type="expression" dxfId="89" priority="24">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A9:C9">
-    <cfRule type="expression" dxfId="75" priority="23">
+    <cfRule type="expression" dxfId="88" priority="23">
       <formula>MOD($A9,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="expression" dxfId="74" priority="22">
+    <cfRule type="expression" dxfId="87" priority="22">
       <formula>MOD($A9,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A10:C10">
-    <cfRule type="expression" dxfId="73" priority="20">
+    <cfRule type="expression" dxfId="86" priority="20">
       <formula>MOD($A10,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D10">
-    <cfRule type="expression" dxfId="72" priority="19">
+    <cfRule type="expression" dxfId="85" priority="19">
       <formula>MOD($A10,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A11:C11">
-    <cfRule type="expression" dxfId="71" priority="18">
+    <cfRule type="expression" dxfId="84" priority="18">
       <formula>MOD($A11,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="expression" dxfId="70" priority="17">
+    <cfRule type="expression" dxfId="83" priority="17">
       <formula>MOD($A11,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A12:C12">
-    <cfRule type="expression" dxfId="69" priority="16">
+    <cfRule type="expression" dxfId="82" priority="16">
       <formula>MOD($A12,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D12">
-    <cfRule type="expression" dxfId="68" priority="15">
+    <cfRule type="expression" dxfId="81" priority="15">
       <formula>MOD($A12,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13:C13">
-    <cfRule type="expression" dxfId="67" priority="14">
+    <cfRule type="expression" dxfId="80" priority="14">
       <formula>MOD($A13,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D13">
-    <cfRule type="expression" dxfId="66" priority="13">
+    <cfRule type="expression" dxfId="79" priority="13">
       <formula>MOD($A13,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14:C14">
-    <cfRule type="expression" dxfId="65" priority="12">
+    <cfRule type="expression" dxfId="78" priority="12">
       <formula>MOD($A14,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D14">
-    <cfRule type="expression" dxfId="64" priority="11">
+    <cfRule type="expression" dxfId="77" priority="11">
       <formula>MOD($A14,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A15:C15">
-    <cfRule type="expression" dxfId="63" priority="10">
+    <cfRule type="expression" dxfId="76" priority="10">
       <formula>MOD($A15,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D15">
-    <cfRule type="expression" dxfId="62" priority="9">
+    <cfRule type="expression" dxfId="75" priority="9">
       <formula>MOD($A15,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:C16">
-    <cfRule type="expression" dxfId="61" priority="8">
+    <cfRule type="expression" dxfId="74" priority="8">
       <formula>MOD($A16,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D16">
-    <cfRule type="expression" dxfId="60" priority="7">
+    <cfRule type="expression" dxfId="73" priority="7">
       <formula>MOD($A16,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A17:C17">
-    <cfRule type="expression" dxfId="59" priority="6">
+    <cfRule type="expression" dxfId="72" priority="6">
       <formula>MOD($A17,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D17">
-    <cfRule type="expression" dxfId="58" priority="5">
+    <cfRule type="expression" dxfId="71" priority="5">
       <formula>MOD($A17,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18:C18">
-    <cfRule type="expression" dxfId="57" priority="4">
+    <cfRule type="expression" dxfId="70" priority="4">
       <formula>MOD($A18,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18">
-    <cfRule type="expression" dxfId="56" priority="3">
+    <cfRule type="expression" dxfId="69" priority="3">
       <formula>MOD($A18,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A19:C19">
-    <cfRule type="expression" dxfId="55" priority="2">
+    <cfRule type="expression" dxfId="68" priority="2">
       <formula>MOD($A19,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D19">
-    <cfRule type="expression" dxfId="54" priority="1">
+    <cfRule type="expression" dxfId="67" priority="1">
       <formula>MOD($A19,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13580,67 +13849,67 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:B62">
-    <cfRule type="expression" dxfId="53" priority="24">
+    <cfRule type="expression" dxfId="66" priority="24">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C8">
-    <cfRule type="expression" dxfId="52" priority="23">
+    <cfRule type="expression" dxfId="65" priority="23">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9">
-    <cfRule type="expression" dxfId="51" priority="21">
+    <cfRule type="expression" dxfId="64" priority="21">
       <formula>MOD($A9,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="expression" dxfId="50" priority="19">
+    <cfRule type="expression" dxfId="63" priority="19">
       <formula>MOD($A10,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11">
-    <cfRule type="expression" dxfId="49" priority="17">
+    <cfRule type="expression" dxfId="62" priority="17">
       <formula>MOD($A11,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C12">
-    <cfRule type="expression" dxfId="48" priority="15">
+    <cfRule type="expression" dxfId="61" priority="15">
       <formula>MOD($A12,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13">
-    <cfRule type="expression" dxfId="47" priority="13">
+    <cfRule type="expression" dxfId="60" priority="13">
       <formula>MOD($A13,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C14">
-    <cfRule type="expression" dxfId="46" priority="11">
+    <cfRule type="expression" dxfId="59" priority="11">
       <formula>MOD($A14,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15">
-    <cfRule type="expression" dxfId="45" priority="9">
+    <cfRule type="expression" dxfId="58" priority="9">
       <formula>MOD($A15,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16">
-    <cfRule type="expression" dxfId="44" priority="7">
+    <cfRule type="expression" dxfId="57" priority="7">
       <formula>MOD($A16,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C17">
-    <cfRule type="expression" dxfId="43" priority="5">
+    <cfRule type="expression" dxfId="56" priority="5">
       <formula>MOD($A17,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18 C20 C22 C24 C26 C28 C30 C32 C34 C36 C38 C40 C42 C44 C46 C48 C50 C52 C54 C56 C58 C60 C62">
-    <cfRule type="expression" dxfId="42" priority="3">
+    <cfRule type="expression" dxfId="55" priority="3">
       <formula>MOD($A18,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19 C21 C23 C25 C27 C29 C31 C33 C35 C37 C39 C41 C43 C45 C47 C49 C51 C53 C55 C57 C59 C61">
-    <cfRule type="expression" dxfId="41" priority="1">
+    <cfRule type="expression" dxfId="54" priority="1">
       <formula>MOD($A19,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16734,6 +17003,429 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:B80 B81">
+    <cfRule type="expression" dxfId="53" priority="13">
+      <formula>MOD($A2,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C8">
+    <cfRule type="expression" dxfId="52" priority="12">
+      <formula>MOD($A2,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9">
+    <cfRule type="expression" dxfId="51" priority="11">
+      <formula>MOD($A9,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10">
+    <cfRule type="expression" dxfId="50" priority="10">
+      <formula>MOD($A10,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11">
+    <cfRule type="expression" dxfId="49" priority="9">
+      <formula>MOD($A11,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C12">
+    <cfRule type="expression" dxfId="48" priority="8">
+      <formula>MOD($A12,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C13">
+    <cfRule type="expression" dxfId="47" priority="7">
+      <formula>MOD($A13,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C14">
+    <cfRule type="expression" dxfId="46" priority="6">
+      <formula>MOD($A14,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C15">
+    <cfRule type="expression" dxfId="45" priority="5">
+      <formula>MOD($A15,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C16">
+    <cfRule type="expression" dxfId="44" priority="4">
+      <formula>MOD($A16,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C17">
+    <cfRule type="expression" dxfId="43" priority="3">
+      <formula>MOD($A17,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C18 C20 C22 C24 C26 C28 C30 C32 C34 C36 C38 C40 C42 C44 C46 C48 C50 C52 C54 C56 C58 C60 C62 C64 C66 C68 C70 C72 C74 C76 C78 C80">
+    <cfRule type="expression" dxfId="42" priority="2">
+      <formula>MOD($A18,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19 C21 C23 C25 C27 C29 C31 C33 C35 C37 C39 C41 C43 C45 C47 C49 C51 C53 C55 C57 C59 C61 C63 C65 C67 C69 C71 C73 C75 C77 C79">
+    <cfRule type="expression" dxfId="41" priority="1">
+      <formula>MOD($A19,2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7C8A748-C354-4D06-9195-40DA5D4F4AE7}">
+  <dimension ref="A1:C38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="75.28515625" style="45" customWidth="1"/>
+    <col min="3" max="3" width="58.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A2" s="13">
+        <v>1</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>1486</v>
+      </c>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A3" s="14">
+        <v>2</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>1487</v>
+      </c>
+      <c r="C3" s="18"/>
+    </row>
+    <row r="4" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A4" s="13">
+        <v>3</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>1488</v>
+      </c>
+      <c r="C4" s="17"/>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="14">
+        <v>4</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>1489</v>
+      </c>
+      <c r="C5" s="18"/>
+    </row>
+    <row r="6" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A6" s="13">
+        <v>5</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>1490</v>
+      </c>
+      <c r="C6" s="17"/>
+    </row>
+    <row r="7" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A7" s="14">
+        <v>6</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>1491</v>
+      </c>
+      <c r="C7" s="18"/>
+    </row>
+    <row r="8" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A8" s="13">
+        <v>7</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C8" s="17"/>
+    </row>
+    <row r="9" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="14">
+        <v>8</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C9" s="18"/>
+    </row>
+    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="35">
+        <v>9</v>
+      </c>
+      <c r="B10" s="42" t="s">
+        <v>1494</v>
+      </c>
+      <c r="C10" s="42"/>
+    </row>
+    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="14">
+        <v>10</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>1495</v>
+      </c>
+      <c r="C11" s="18"/>
+    </row>
+    <row r="12" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A12" s="13">
+        <v>11</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>1496</v>
+      </c>
+      <c r="C12" s="17"/>
+    </row>
+    <row r="13" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A13" s="14">
+        <v>12</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C13" s="18"/>
+    </row>
+    <row r="14" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A14" s="13">
+        <v>13</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>1498</v>
+      </c>
+      <c r="C14" s="17"/>
+    </row>
+    <row r="15" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A15" s="14">
+        <v>14</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>1499</v>
+      </c>
+      <c r="C15" s="18"/>
+    </row>
+    <row r="16" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="13">
+        <v>15</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>1500</v>
+      </c>
+      <c r="C16" s="17"/>
+    </row>
+    <row r="17" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="14">
+        <v>16</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>1501</v>
+      </c>
+      <c r="C17" s="18"/>
+    </row>
+    <row r="18" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A18" s="13">
+        <v>17</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>1502</v>
+      </c>
+      <c r="C18" s="17"/>
+    </row>
+    <row r="19" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A19" s="14">
+        <v>18</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>1503</v>
+      </c>
+      <c r="C19" s="18"/>
+    </row>
+    <row r="20" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="13">
+        <v>19</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C20" s="17"/>
+    </row>
+    <row r="21" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A21" s="14">
+        <v>20</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>1505</v>
+      </c>
+      <c r="C21" s="18"/>
+    </row>
+    <row r="22" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A22" s="13">
+        <v>21</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>1506</v>
+      </c>
+      <c r="C22" s="17"/>
+    </row>
+    <row r="23" spans="1:3" ht="66" x14ac:dyDescent="0.25">
+      <c r="A23" s="14">
+        <v>22</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C23" s="18"/>
+    </row>
+    <row r="24" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A24" s="13">
+        <v>23</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>1508</v>
+      </c>
+      <c r="C24" s="17"/>
+    </row>
+    <row r="25" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="14">
+        <v>24</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>1509</v>
+      </c>
+      <c r="C25" s="18"/>
+    </row>
+    <row r="26" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A26" s="13">
+        <v>25</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C26" s="17"/>
+    </row>
+    <row r="27" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A27" s="14">
+        <v>26</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>1511</v>
+      </c>
+      <c r="C27" s="18"/>
+    </row>
+    <row r="28" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A28" s="13">
+        <v>27</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C28" s="17"/>
+    </row>
+    <row r="29" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="14">
+        <v>28</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>1513</v>
+      </c>
+      <c r="C29" s="18"/>
+    </row>
+    <row r="30" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A30" s="13">
+        <v>29</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>1514</v>
+      </c>
+      <c r="C30" s="17"/>
+    </row>
+    <row r="31" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="14">
+        <v>30</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>1515</v>
+      </c>
+      <c r="C31" s="18"/>
+    </row>
+    <row r="32" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="13">
+        <v>31</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>1516</v>
+      </c>
+      <c r="C32" s="17"/>
+    </row>
+    <row r="33" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A33" s="14">
+        <v>32</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>1517</v>
+      </c>
+      <c r="C33" s="18"/>
+    </row>
+    <row r="34" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A34" s="13">
+        <v>33</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>1518</v>
+      </c>
+      <c r="C34" s="17"/>
+    </row>
+    <row r="35" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="14">
+        <v>34</v>
+      </c>
+      <c r="B35" s="18" t="s">
+        <v>1519</v>
+      </c>
+      <c r="C35" s="18"/>
+    </row>
+    <row r="36" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="13">
+        <v>35</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>1520</v>
+      </c>
+      <c r="C36" s="17"/>
+    </row>
+    <row r="37" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A37" s="14">
+        <v>36</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>1521</v>
+      </c>
+      <c r="C37" s="18"/>
+    </row>
+    <row r="38" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A38" s="13">
+        <v>37</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>1522</v>
+      </c>
+      <c r="C38" s="17"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C38 A2:B38">
     <cfRule type="expression" dxfId="40" priority="13">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
@@ -16788,12 +17480,12 @@
       <formula>MOD($A17,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C18 C20 C22 C24 C26 C28 C30 C32 C34 C36 C38 C40 C42 C44 C46 C48 C50 C52 C54 C56 C58 C60 C62 C64 C66 C68 C70 C72 C74 C76 C78 C80">
+  <conditionalFormatting sqref="C18 C20 C22 C24 C26 C28 C30 C32 C34 C36">
     <cfRule type="expression" dxfId="29" priority="2">
       <formula>MOD($A18,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C19 C21 C23 C25 C27 C29 C31 C33 C35 C37 C39 C41 C43 C45 C47 C49 C51 C53 C55 C57 C59 C61 C63 C65 C67 C69 C71 C73 C75 C77 C79">
+  <conditionalFormatting sqref="C19 C21 C23 C25 C27 C29 C31 C33 C35 C37">
     <cfRule type="expression" dxfId="28" priority="1">
       <formula>MOD($A19,2)=0</formula>
     </cfRule>
@@ -16802,9 +17494,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7C8A748-C354-4D06-9195-40DA5D4F4AE7}">
-  <dimension ref="A1:C38"/>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB27444-2806-457F-A982-2305DF913562}">
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="75.28515625" style="45" customWidth="1"/>
@@ -16822,12 +17514,12 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="13">
         <v>1</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>1486</v>
+        <v>1523</v>
       </c>
       <c r="C2" s="17"/>
     </row>
@@ -16836,16 +17528,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>1487</v>
+        <v>1524</v>
       </c>
       <c r="C3" s="18"/>
     </row>
-    <row r="4" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4" s="13">
         <v>3</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>1488</v>
+        <v>1525</v>
       </c>
       <c r="C4" s="17"/>
     </row>
@@ -16854,7 +17546,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>1489</v>
+        <v>1526</v>
       </c>
       <c r="C5" s="18"/>
     </row>
@@ -16863,34 +17555,34 @@
         <v>5</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>1490</v>
+        <v>1527</v>
       </c>
       <c r="C6" s="17"/>
     </row>
-    <row r="7" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7" s="14">
         <v>6</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>1491</v>
+        <v>1528</v>
       </c>
       <c r="C7" s="18"/>
     </row>
-    <row r="8" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A8" s="13">
         <v>7</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>1492</v>
+        <v>1529</v>
       </c>
       <c r="C8" s="17"/>
     </row>
-    <row r="9" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" s="14">
         <v>8</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>1493</v>
+        <v>1530</v>
       </c>
       <c r="C9" s="18"/>
     </row>
@@ -16899,7 +17591,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="42" t="s">
-        <v>1494</v>
+        <v>1531</v>
       </c>
       <c r="C10" s="42"/>
     </row>
@@ -16908,7 +17600,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>1495</v>
+        <v>1532</v>
       </c>
       <c r="C11" s="18"/>
     </row>
@@ -16917,43 +17609,43 @@
         <v>11</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>1496</v>
+        <v>1533</v>
       </c>
       <c r="C12" s="17"/>
     </row>
-    <row r="13" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A13" s="14">
         <v>12</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>1497</v>
+        <v>1534</v>
       </c>
       <c r="C13" s="18"/>
     </row>
-    <row r="14" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A14" s="13">
         <v>13</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>1498</v>
+        <v>1535</v>
       </c>
       <c r="C14" s="17"/>
     </row>
-    <row r="15" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A15" s="14">
         <v>14</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>1499</v>
+        <v>1536</v>
       </c>
       <c r="C15" s="18"/>
     </row>
-    <row r="16" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A16" s="13">
         <v>15</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>1500</v>
+        <v>1537</v>
       </c>
       <c r="C16" s="17"/>
     </row>
@@ -16962,7 +17654,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>1501</v>
+        <v>1538</v>
       </c>
       <c r="C17" s="18"/>
     </row>
@@ -16971,16 +17663,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>1502</v>
+        <v>1539</v>
       </c>
       <c r="C18" s="17"/>
     </row>
-    <row r="19" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A19" s="14">
         <v>18</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>1503</v>
+        <v>1540</v>
       </c>
       <c r="C19" s="18"/>
     </row>
@@ -16989,16 +17681,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>1504</v>
+        <v>1541</v>
       </c>
       <c r="C20" s="17"/>
     </row>
-    <row r="21" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A21" s="14">
         <v>20</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>1505</v>
+        <v>895</v>
       </c>
       <c r="C21" s="18"/>
     </row>
@@ -17007,79 +17699,79 @@
         <v>21</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>1506</v>
+        <v>1542</v>
       </c>
       <c r="C22" s="17"/>
     </row>
-    <row r="23" spans="1:3" ht="66" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A23" s="14">
         <v>22</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>1507</v>
+        <v>1543</v>
       </c>
       <c r="C23" s="18"/>
     </row>
-    <row r="24" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A24" s="13">
         <v>23</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>1508</v>
+        <v>1544</v>
       </c>
       <c r="C24" s="17"/>
     </row>
-    <row r="25" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A25" s="14">
         <v>24</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>1509</v>
+        <v>1545</v>
       </c>
       <c r="C25" s="18"/>
     </row>
-    <row r="26" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A26" s="13">
         <v>25</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>1510</v>
+        <v>1546</v>
       </c>
       <c r="C26" s="17"/>
     </row>
-    <row r="27" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A27" s="14">
         <v>26</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>1511</v>
+        <v>1547</v>
       </c>
       <c r="C27" s="18"/>
     </row>
-    <row r="28" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A28" s="13">
         <v>27</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>1512</v>
+        <v>1548</v>
       </c>
       <c r="C28" s="17"/>
     </row>
-    <row r="29" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A29" s="14">
         <v>28</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>1513</v>
+        <v>1549</v>
       </c>
       <c r="C29" s="18"/>
     </row>
-    <row r="30" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A30" s="13">
         <v>29</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>1514</v>
+        <v>1550</v>
       </c>
       <c r="C30" s="17"/>
     </row>
@@ -17088,16 +17780,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>1515</v>
+        <v>1551</v>
       </c>
       <c r="C31" s="18"/>
     </row>
-    <row r="32" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A32" s="13">
         <v>31</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>1516</v>
+        <v>1552</v>
       </c>
       <c r="C32" s="17"/>
     </row>
@@ -17106,25 +17798,25 @@
         <v>32</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>1517</v>
+        <v>1553</v>
       </c>
       <c r="C33" s="18"/>
     </row>
-    <row r="34" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A34" s="13">
         <v>33</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>1518</v>
+        <v>1554</v>
       </c>
       <c r="C34" s="17"/>
     </row>
-    <row r="35" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A35" s="14">
         <v>34</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>1519</v>
+        <v>1555</v>
       </c>
       <c r="C35" s="18"/>
     </row>
@@ -17133,16 +17825,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>1520</v>
+        <v>1556</v>
       </c>
       <c r="C36" s="17"/>
     </row>
-    <row r="37" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A37" s="14">
         <v>36</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>1521</v>
+        <v>1557</v>
       </c>
       <c r="C37" s="18"/>
     </row>
@@ -17151,12 +17843,318 @@
         <v>37</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>1522</v>
+        <v>1558</v>
       </c>
       <c r="C38" s="17"/>
     </row>
+    <row r="39" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A39" s="13">
+        <v>38</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>1559</v>
+      </c>
+      <c r="C39" s="17"/>
+    </row>
+    <row r="40" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A40" s="14">
+        <v>39</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>1560</v>
+      </c>
+      <c r="C40" s="18"/>
+    </row>
+    <row r="41" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A41" s="13">
+        <v>40</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>1561</v>
+      </c>
+      <c r="C41" s="17"/>
+    </row>
+    <row r="42" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A42" s="13">
+        <v>41</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>1562</v>
+      </c>
+      <c r="C42" s="17"/>
+    </row>
+    <row r="43" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A43" s="14">
+        <v>42</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>1563</v>
+      </c>
+      <c r="C43" s="18"/>
+    </row>
+    <row r="44" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A44" s="13">
+        <v>43</v>
+      </c>
+      <c r="B44" s="17" t="s">
+        <v>1564</v>
+      </c>
+      <c r="C44" s="17"/>
+    </row>
+    <row r="45" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A45" s="13">
+        <v>44</v>
+      </c>
+      <c r="B45" s="17" t="s">
+        <v>1565</v>
+      </c>
+      <c r="C45" s="17"/>
+    </row>
+    <row r="46" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A46" s="14">
+        <v>45</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>1566</v>
+      </c>
+      <c r="C46" s="18"/>
+    </row>
+    <row r="47" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A47" s="13">
+        <v>46</v>
+      </c>
+      <c r="B47" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="C47" s="17"/>
+    </row>
+    <row r="48" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A48" s="13">
+        <v>47</v>
+      </c>
+      <c r="B48" s="17" t="s">
+        <v>1567</v>
+      </c>
+      <c r="C48" s="17"/>
+    </row>
+    <row r="49" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A49" s="14">
+        <v>48</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>1568</v>
+      </c>
+      <c r="C49" s="18"/>
+    </row>
+    <row r="50" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="13">
+        <v>49</v>
+      </c>
+      <c r="B50" s="17" t="s">
+        <v>1569</v>
+      </c>
+      <c r="C50" s="17"/>
+    </row>
+    <row r="51" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A51" s="13">
+        <v>50</v>
+      </c>
+      <c r="B51" s="17" t="s">
+        <v>1570</v>
+      </c>
+      <c r="C51" s="17"/>
+    </row>
+    <row r="52" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A52" s="14">
+        <v>51</v>
+      </c>
+      <c r="B52" s="18" t="s">
+        <v>1571</v>
+      </c>
+      <c r="C52" s="18"/>
+    </row>
+    <row r="53" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A53" s="13">
+        <v>52</v>
+      </c>
+      <c r="B53" s="17" t="s">
+        <v>1572</v>
+      </c>
+      <c r="C53" s="17"/>
+    </row>
+    <row r="54" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A54" s="13">
+        <v>53</v>
+      </c>
+      <c r="B54" s="17" t="s">
+        <v>1573</v>
+      </c>
+      <c r="C54" s="17"/>
+    </row>
+    <row r="55" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A55" s="14">
+        <v>54</v>
+      </c>
+      <c r="B55" s="18" t="s">
+        <v>1574</v>
+      </c>
+      <c r="C55" s="18"/>
+    </row>
+    <row r="56" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A56" s="13">
+        <v>55</v>
+      </c>
+      <c r="B56" s="17" t="s">
+        <v>1575</v>
+      </c>
+      <c r="C56" s="17"/>
+    </row>
+    <row r="57" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A57" s="13">
+        <v>56</v>
+      </c>
+      <c r="B57" s="17" t="s">
+        <v>1576</v>
+      </c>
+      <c r="C57" s="17"/>
+    </row>
+    <row r="58" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A58" s="14">
+        <v>57</v>
+      </c>
+      <c r="B58" s="18" t="s">
+        <v>1577</v>
+      </c>
+      <c r="C58" s="18"/>
+    </row>
+    <row r="59" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A59" s="13">
+        <v>58</v>
+      </c>
+      <c r="B59" s="17" t="s">
+        <v>1578</v>
+      </c>
+      <c r="C59" s="17"/>
+    </row>
+    <row r="60" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A60" s="13">
+        <v>59</v>
+      </c>
+      <c r="B60" s="17" t="s">
+        <v>1579</v>
+      </c>
+      <c r="C60" s="17"/>
+    </row>
+    <row r="61" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="14">
+        <v>60</v>
+      </c>
+      <c r="B61" s="18" t="s">
+        <v>1580</v>
+      </c>
+      <c r="C61" s="18"/>
+    </row>
+    <row r="62" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A62" s="13">
+        <v>61</v>
+      </c>
+      <c r="B62" s="17" t="s">
+        <v>1581</v>
+      </c>
+      <c r="C62" s="17"/>
+    </row>
+    <row r="63" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="13">
+        <v>62</v>
+      </c>
+      <c r="B63" s="17" t="s">
+        <v>1582</v>
+      </c>
+      <c r="C63" s="17"/>
+    </row>
+    <row r="64" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A64" s="14">
+        <v>63</v>
+      </c>
+      <c r="B64" s="18" t="s">
+        <v>1583</v>
+      </c>
+      <c r="C64" s="18"/>
+    </row>
+    <row r="65" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A65" s="13">
+        <v>64</v>
+      </c>
+      <c r="B65" s="17" t="s">
+        <v>1584</v>
+      </c>
+      <c r="C65" s="17"/>
+    </row>
+    <row r="66" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A66" s="13">
+        <v>65</v>
+      </c>
+      <c r="B66" s="17" t="s">
+        <v>1585</v>
+      </c>
+      <c r="C66" s="17"/>
+    </row>
+    <row r="67" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A67" s="14">
+        <v>66</v>
+      </c>
+      <c r="B67" s="18" t="s">
+        <v>1586</v>
+      </c>
+      <c r="C67" s="18"/>
+    </row>
+    <row r="68" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A68" s="13">
+        <v>67</v>
+      </c>
+      <c r="B68" s="17" t="s">
+        <v>1587</v>
+      </c>
+      <c r="C68" s="17"/>
+    </row>
+    <row r="69" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A69" s="13">
+        <v>68</v>
+      </c>
+      <c r="B69" s="17" t="s">
+        <v>1588</v>
+      </c>
+      <c r="C69" s="17"/>
+    </row>
+    <row r="70" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+      <c r="A70" s="14">
+        <v>69</v>
+      </c>
+      <c r="B70" s="18" t="s">
+        <v>1589</v>
+      </c>
+      <c r="C70" s="18"/>
+    </row>
+    <row r="71" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A71" s="13">
+        <v>70</v>
+      </c>
+      <c r="B71" s="17" t="s">
+        <v>1590</v>
+      </c>
+      <c r="C71" s="17"/>
+    </row>
+    <row r="72" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A72" s="13">
+        <v>71</v>
+      </c>
+      <c r="B72" s="17" t="s">
+        <v>1591</v>
+      </c>
+      <c r="C72" s="17"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C38 A2:B38">
+  <conditionalFormatting sqref="C38 C41 C44 C47 C50 C53 C56 C59 C62 C65 C68 C71 A2:B72">
     <cfRule type="expression" dxfId="27" priority="13">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
@@ -17211,12 +18209,12 @@
       <formula>MOD($A17,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C18 C20 C22 C24 C26 C28 C30 C32 C34 C36">
+  <conditionalFormatting sqref="C18 C20 C22 C24 C26 C28 C30 C32 C34 C36 C39 C42 C45 C48 C51 C54 C57 C60 C63 C66 C69 C72">
     <cfRule type="expression" dxfId="16" priority="2">
       <formula>MOD($A18,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C19 C21 C23 C25 C27 C29 C31 C33 C35 C37">
+  <conditionalFormatting sqref="C19 C21 C23 C25 C27 C29 C31 C33 C35 C37 C40 C43 C46 C49 C52 C55 C58 C61 C64 C67 C70">
     <cfRule type="expression" dxfId="15" priority="1">
       <formula>MOD($A19,2)=0</formula>
     </cfRule>
@@ -17225,13 +18223,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB27444-2806-457F-A982-2305DF913562}">
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6BD4D45-6E6B-42C6-B19B-4190FAC45CF0}">
   <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="75.28515625" style="45" customWidth="1"/>
-    <col min="3" max="3" width="58.28515625" customWidth="1"/>
+    <col min="2" max="2" width="57.7109375" customWidth="1"/>
+    <col min="3" max="3" width="68.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -17245,12 +18243,12 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A2" s="13">
         <v>1</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>1523</v>
+        <v>1592</v>
       </c>
       <c r="C2" s="17"/>
     </row>
@@ -17259,7 +18257,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>1524</v>
+        <v>1593</v>
       </c>
       <c r="C3" s="18"/>
     </row>
@@ -17268,16 +18266,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>1525</v>
+        <v>1594</v>
       </c>
       <c r="C4" s="17"/>
     </row>
-    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A5" s="14">
         <v>4</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>1526</v>
+        <v>1595</v>
       </c>
       <c r="C5" s="18"/>
     </row>
@@ -17286,7 +18284,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>1527</v>
+        <v>1596</v>
       </c>
       <c r="C6" s="17"/>
     </row>
@@ -17295,16 +18293,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>1528</v>
+        <v>1597</v>
       </c>
       <c r="C7" s="18"/>
     </row>
-    <row r="8" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="66" x14ac:dyDescent="0.25">
       <c r="A8" s="13">
         <v>7</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>1529</v>
+        <v>1598</v>
       </c>
       <c r="C8" s="17"/>
     </row>
@@ -17313,16 +18311,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>1530</v>
+        <v>1599</v>
       </c>
       <c r="C9" s="18"/>
     </row>
-    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A10" s="35">
         <v>9</v>
       </c>
       <c r="B10" s="42" t="s">
-        <v>1531</v>
+        <v>1600</v>
       </c>
       <c r="C10" s="42"/>
     </row>
@@ -17331,25 +18329,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>1532</v>
+        <v>1601</v>
       </c>
       <c r="C11" s="18"/>
     </row>
-    <row r="12" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A12" s="13">
         <v>11</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>1533</v>
+        <v>1602</v>
       </c>
       <c r="C12" s="17"/>
     </row>
-    <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A13" s="14">
         <v>12</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>1534</v>
+        <v>1603</v>
       </c>
       <c r="C13" s="18"/>
     </row>
@@ -17358,7 +18356,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>1535</v>
+        <v>1604</v>
       </c>
       <c r="C14" s="17"/>
     </row>
@@ -17367,7 +18365,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>1536</v>
+        <v>1605</v>
       </c>
       <c r="C15" s="18"/>
     </row>
@@ -17376,7 +18374,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>1537</v>
+        <v>1606</v>
       </c>
       <c r="C16" s="17"/>
     </row>
@@ -17385,61 +18383,61 @@
         <v>16</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>1538</v>
+        <v>1607</v>
       </c>
       <c r="C17" s="18"/>
     </row>
-    <row r="18" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A18" s="13">
         <v>17</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>1539</v>
+        <v>1608</v>
       </c>
       <c r="C18" s="17"/>
     </row>
-    <row r="19" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A19" s="14">
         <v>18</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>1540</v>
+        <v>1609</v>
       </c>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A20" s="13">
         <v>19</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>1541</v>
+        <v>1610</v>
       </c>
       <c r="C20" s="17"/>
     </row>
-    <row r="21" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A21" s="14">
         <v>20</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>895</v>
+        <v>1611</v>
       </c>
       <c r="C21" s="18"/>
     </row>
-    <row r="22" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A22" s="13">
         <v>21</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>1542</v>
+        <v>1612</v>
       </c>
       <c r="C22" s="17"/>
     </row>
-    <row r="23" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A23" s="14">
         <v>22</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>1543</v>
+        <v>1613</v>
       </c>
       <c r="C23" s="18"/>
     </row>
@@ -17448,7 +18446,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>1544</v>
+        <v>1614</v>
       </c>
       <c r="C24" s="17"/>
     </row>
@@ -17457,16 +18455,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>1545</v>
+        <v>1615</v>
       </c>
       <c r="C25" s="18"/>
     </row>
-    <row r="26" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A26" s="13">
         <v>25</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>1546</v>
+        <v>1616</v>
       </c>
       <c r="C26" s="17"/>
     </row>
@@ -17475,7 +18473,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>1547</v>
+        <v>1617</v>
       </c>
       <c r="C27" s="18"/>
     </row>
@@ -17484,16 +18482,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>1548</v>
+        <v>1618</v>
       </c>
       <c r="C28" s="17"/>
     </row>
-    <row r="29" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A29" s="14">
         <v>28</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>1549</v>
+        <v>1619</v>
       </c>
       <c r="C29" s="18"/>
     </row>
@@ -17502,34 +18500,34 @@
         <v>29</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>1550</v>
+        <v>1620</v>
       </c>
       <c r="C30" s="17"/>
     </row>
-    <row r="31" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A31" s="14">
         <v>30</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>1551</v>
+        <v>1621</v>
       </c>
       <c r="C31" s="18"/>
     </row>
-    <row r="32" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A32" s="13">
         <v>31</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>1552</v>
+        <v>1622</v>
       </c>
       <c r="C32" s="17"/>
     </row>
-    <row r="33" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A33" s="14">
         <v>32</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>1553</v>
+        <v>1623</v>
       </c>
       <c r="C33" s="18"/>
     </row>
@@ -17538,7 +18536,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>1554</v>
+        <v>1624</v>
       </c>
       <c r="C34" s="17"/>
     </row>
@@ -17547,7 +18545,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>1555</v>
+        <v>1625</v>
       </c>
       <c r="C35" s="18"/>
     </row>
@@ -17556,7 +18554,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>1556</v>
+        <v>1626</v>
       </c>
       <c r="C36" s="17"/>
     </row>
@@ -17565,7 +18563,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>1557</v>
+        <v>1627</v>
       </c>
       <c r="C37" s="18"/>
     </row>
@@ -17574,16 +18572,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>1558</v>
+        <v>1628</v>
       </c>
       <c r="C38" s="17"/>
     </row>
-    <row r="39" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A39" s="13">
         <v>38</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>1559</v>
+        <v>1629</v>
       </c>
       <c r="C39" s="17"/>
     </row>
@@ -17592,7 +18590,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>1560</v>
+        <v>1630</v>
       </c>
       <c r="C40" s="18"/>
     </row>
@@ -17601,16 +18599,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>1561</v>
+        <v>1631</v>
       </c>
       <c r="C41" s="17"/>
     </row>
-    <row r="42" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A42" s="13">
         <v>41</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>1562</v>
+        <v>1632</v>
       </c>
       <c r="C42" s="17"/>
     </row>
@@ -17619,7 +18617,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="18" t="s">
-        <v>1563</v>
+        <v>1633</v>
       </c>
       <c r="C43" s="18"/>
     </row>
@@ -17628,16 +18626,16 @@
         <v>43</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>1564</v>
+        <v>1634</v>
       </c>
       <c r="C44" s="17"/>
     </row>
-    <row r="45" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A45" s="13">
         <v>44</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>1565</v>
+        <v>1635</v>
       </c>
       <c r="C45" s="17"/>
     </row>
@@ -17646,7 +18644,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>1566</v>
+        <v>619</v>
       </c>
       <c r="C46" s="18"/>
     </row>
@@ -17655,16 +18653,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>155</v>
+        <v>1636</v>
       </c>
       <c r="C47" s="17"/>
     </row>
-    <row r="48" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A48" s="13">
         <v>47</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>1567</v>
+        <v>1637</v>
       </c>
       <c r="C48" s="17"/>
     </row>
@@ -17673,7 +18671,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>1568</v>
+        <v>1638</v>
       </c>
       <c r="C49" s="18"/>
     </row>
@@ -17682,7 +18680,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="17" t="s">
-        <v>1569</v>
+        <v>1639</v>
       </c>
       <c r="C50" s="17"/>
     </row>
@@ -17691,7 +18689,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>1570</v>
+        <v>1640</v>
       </c>
       <c r="C51" s="17"/>
     </row>
@@ -17700,7 +18698,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="18" t="s">
-        <v>1571</v>
+        <v>1641</v>
       </c>
       <c r="C52" s="18"/>
     </row>
@@ -17709,16 +18707,16 @@
         <v>52</v>
       </c>
       <c r="B53" s="17" t="s">
-        <v>1572</v>
+        <v>1642</v>
       </c>
       <c r="C53" s="17"/>
     </row>
-    <row r="54" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A54" s="13">
         <v>53</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>1573</v>
+        <v>1643</v>
       </c>
       <c r="C54" s="17"/>
     </row>
@@ -17727,43 +18725,43 @@
         <v>54</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>1574</v>
+        <v>1644</v>
       </c>
       <c r="C55" s="18"/>
     </row>
-    <row r="56" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A56" s="13">
         <v>55</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>1575</v>
+        <v>1645</v>
       </c>
       <c r="C56" s="17"/>
     </row>
-    <row r="57" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A57" s="13">
         <v>56</v>
       </c>
       <c r="B57" s="17" t="s">
-        <v>1576</v>
+        <v>1646</v>
       </c>
       <c r="C57" s="17"/>
     </row>
-    <row r="58" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A58" s="14">
         <v>57</v>
       </c>
       <c r="B58" s="18" t="s">
-        <v>1577</v>
+        <v>1647</v>
       </c>
       <c r="C58" s="18"/>
     </row>
-    <row r="59" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" ht="33" x14ac:dyDescent="0.25">
       <c r="A59" s="13">
         <v>58</v>
       </c>
       <c r="B59" s="17" t="s">
-        <v>1578</v>
+        <v>1648</v>
       </c>
       <c r="C59" s="17"/>
     </row>
@@ -17772,7 +18770,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="17" t="s">
-        <v>1579</v>
+        <v>1649</v>
       </c>
       <c r="C60" s="17"/>
     </row>
@@ -17781,7 +18779,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="18" t="s">
-        <v>1580</v>
+        <v>1650</v>
       </c>
       <c r="C61" s="18"/>
     </row>
@@ -17790,7 +18788,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="17" t="s">
-        <v>1581</v>
+        <v>1631</v>
       </c>
       <c r="C62" s="17"/>
     </row>
@@ -17798,155 +18796,135 @@
       <c r="A63" s="13">
         <v>62</v>
       </c>
-      <c r="B63" s="17" t="s">
-        <v>1582</v>
-      </c>
+      <c r="B63" s="17"/>
       <c r="C63" s="17"/>
     </row>
     <row r="64" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A64" s="14">
         <v>63</v>
       </c>
-      <c r="B64" s="18" t="s">
-        <v>1583</v>
-      </c>
+      <c r="B64" s="18"/>
       <c r="C64" s="18"/>
     </row>
     <row r="65" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A65" s="13">
         <v>64</v>
       </c>
-      <c r="B65" s="17" t="s">
-        <v>1584</v>
-      </c>
+      <c r="B65" s="17"/>
       <c r="C65" s="17"/>
     </row>
     <row r="66" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A66" s="13">
         <v>65</v>
       </c>
-      <c r="B66" s="17" t="s">
-        <v>1585</v>
-      </c>
+      <c r="B66" s="17"/>
       <c r="C66" s="17"/>
     </row>
     <row r="67" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A67" s="14">
         <v>66</v>
       </c>
-      <c r="B67" s="18" t="s">
-        <v>1586</v>
-      </c>
+      <c r="B67" s="18"/>
       <c r="C67" s="18"/>
     </row>
-    <row r="68" spans="1:3" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A68" s="13">
         <v>67</v>
       </c>
-      <c r="B68" s="17" t="s">
-        <v>1587</v>
-      </c>
+      <c r="B68" s="17"/>
       <c r="C68" s="17"/>
     </row>
     <row r="69" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A69" s="13">
         <v>68</v>
       </c>
-      <c r="B69" s="17" t="s">
-        <v>1588</v>
-      </c>
+      <c r="B69" s="17"/>
       <c r="C69" s="17"/>
     </row>
-    <row r="70" spans="1:3" ht="33" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A70" s="14">
         <v>69</v>
       </c>
-      <c r="B70" s="18" t="s">
-        <v>1589</v>
-      </c>
+      <c r="B70" s="18"/>
       <c r="C70" s="18"/>
     </row>
     <row r="71" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A71" s="13">
         <v>70</v>
       </c>
-      <c r="B71" s="17" t="s">
-        <v>1590</v>
-      </c>
+      <c r="B71" s="17"/>
       <c r="C71" s="17"/>
     </row>
     <row r="72" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A72" s="13">
         <v>71</v>
       </c>
-      <c r="B72" s="17" t="s">
-        <v>1591</v>
-      </c>
+      <c r="B72" s="17"/>
       <c r="C72" s="17"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C38 C41 C44 C47 C50 C53 C56 C59 C62 C65 C68 C71 A2:B72">
-    <cfRule type="expression" dxfId="14" priority="13">
+    <cfRule type="expression" dxfId="12" priority="13">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C8">
-    <cfRule type="expression" dxfId="13" priority="12">
+    <cfRule type="expression" dxfId="11" priority="12">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9">
-    <cfRule type="expression" dxfId="12" priority="11">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>MOD($A9,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="expression" dxfId="11" priority="10">
+    <cfRule type="expression" dxfId="9" priority="10">
       <formula>MOD($A10,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11">
-    <cfRule type="expression" dxfId="10" priority="9">
+    <cfRule type="expression" dxfId="8" priority="9">
       <formula>MOD($A11,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C12">
-    <cfRule type="expression" dxfId="9" priority="8">
+    <cfRule type="expression" dxfId="7" priority="8">
       <formula>MOD($A12,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13">
-    <cfRule type="expression" dxfId="8" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>MOD($A13,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C14">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>MOD($A14,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15">
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>MOD($A15,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16">
-    <cfRule type="expression" dxfId="5" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>MOD($A16,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C17">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>MOD($A17,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18 C20 C22 C24 C26 C28 C30 C32 C34 C36 C39 C42 C45 C48 C51 C54 C57 C60 C63 C66 C69 C72">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>MOD($A18,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19 C21 C23 C25 C27 C29 C31 C33 C35 C37 C40 C43 C46 C49 C52 C55 C58 C61 C64 C67 C70">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>MOD($A19,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17954,7 +18932,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C151D989-7212-4279-BDF6-FF7D25CBFE06}">
   <dimension ref="A1:G131"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
@@ -19303,12 +20281,12 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:G1048576">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19317,7 +20295,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B37D5207-7F73-4E5C-BE8D-0639D4780A4C}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
@@ -19419,7 +20397,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD3A1EF4-C67F-44C5-AF2E-C90C930721E1}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
@@ -19523,7 +20501,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAD48A54-82F9-4DF6-887D-71F3D4BD6A2F}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
@@ -19707,7 +20685,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4B18F70-0222-49B3-A1BC-D35362C5AAFC}">
   <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -21557,7 +22535,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="93" priority="1">
+    <cfRule type="expression" dxfId="106" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -22363,7 +23341,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="92" priority="1">
+    <cfRule type="expression" dxfId="105" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -23203,7 +24181,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="91" priority="1">
+    <cfRule type="expression" dxfId="104" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -24235,7 +25213,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="90" priority="1">
+    <cfRule type="expression" dxfId="103" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25055,7 +26033,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="89" priority="1">
+    <cfRule type="expression" dxfId="102" priority="1">
       <formula>MOD($A2,2)=0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>